<commit_message>
fix(extraction): khoản/điều có ngày hiệu lực riêng mang đúng ngày đó
- extract_provision_events.py đọc câu "Các khoản 4, ... 12 Điều 1 Thông tư
  này có hiệu lực từ ngày ..." ngoài phần trích dẫn, gán ngày cho sự kiện
  nằm trong khoản/điều đó thay vì ngày của cả văn bản (D5 §5.1). Bỏ qua câu
  chỉ hẹn ngày cho một phần nội dung hoặc nêu Điểm. Chạy thử: 160 sự kiện
  của 26 văn bản đổi ngày, 75 được áp; chưa dựng lại (W2-09).
- Phiếu audit T1/T2/T3/T6 thêm đoạn trích văn bản gốc và văn bản tác động
  cho 468 dòng; crosscheck_evidence.py chịu dòng không có số Điều.
- ADR 0004: amendment §4 cho model embedding PhoBERT, không qua Milvus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/review/audit_T1.xlsx
+++ b/data/review/audit_T1.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007F3F00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,8 +429,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W56"/>
+  <dimension ref="A1:Y56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="24" max="24"/>
+    <col width="80" customWidth="1" min="25" max="25"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -532,6 +552,16 @@
           <t>audit_note</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>trich_van_ban_goc</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>trich_van_ban_tac_dong</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -584,9 +614,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=19196</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -597,7 +624,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>valid_to_wrong</t>
@@ -608,11 +634,25 @@
           <t>NĐ 161/2004/NĐ-CP đã bị NĐ 36/2007/NĐ-CP (xử phạt VPHC lĩnh vực chứng khoán) thay thế; valid_to vẫn rỗng; id cũ vilextime:T1:provision:0874e970-3425-11f1-9e65-619eaa3c24f9:2004-10-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>161/2004/NĐ-CP · hiệu lực 2004-10-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 8. Xử phạt đối với những hành vi vi phạm các quy định về phát hành chứng khoán ra công chúng
+1. Phạt tiền từ 10.000.000 đồng đến 20.000.000 đồng đối với mỗi tổ chức phát hành, tổ chức tư vấn phát hành thực hiện một trong những hành vi vi phạm sau:
+a) Hồ sơ đăng ký phát hành chứng khoán ra công chúng gửi Uỷ ban Chứng khoán Nhà nước có thông tin sai lệch hoặc che dấu sự thật;
+b) Sử dụng các thông tin ngoài bản cáo bạch để thăm dò thị trường trước khi được phép phát hành chứng khoán ra công chúng;
+c) Phân phối chứng khoán ra công chúng trước khi thực hiện việc công bố phát hành;
+d) Phát hành chứng khoán ra công chúng không theo đúng nội dung đăng ký phát hành về chủng loại chứng khoán, thời hạn phát hành và khối lượng tối thiểu theo quy định;
+đ) Thông báo phát hành chứng khoán trên các phương tiện thông tin đại chúng không đúng nội dung, thời hạn và thời gian theo quy định;
+e) Không có tổ chức trung gian tài chính tham gia bảo lãnh phát hành đối với trường hợp phát hành trái phiếu;
+g) Tổ chức bảo lãnh phát hành thực hiện bảo lãnh phát hành tổng giá trị chứng khoán vượt quá tỷ lệ quy định của pháp luật.</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -665,9 +705,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=13896</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -678,7 +715,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -689,11 +725,17 @@
           <t>Mục 2.9.c bị ghi thành 'Điểm c Khoản 2'; id cũ vilextime:T1:provision:09e3e960-2759-11f1-aa6b-33c42ee76deb:2007-08-08: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>72/2007/TT-BTC · hiệu lực 2007-08-07 → 2017-01-01 · lúc thu thập: Hết hiệu lực toàn bộ
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -746,9 +788,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=183370</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -759,18 +798,38 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trong lĩnh vực chức danh nghề nghiệp bác sĩ y học dự phòng, nhiệm vụ về truyền thông giáo dục sức khỏe và quản lý sức khỏe cộng đồng gồm những việc gì?»; nhãn cũ khong_dat question_ambiguous: Thông tư có ba Điều cho ba hạng bác sĩ y học dự phòng (Điều 7 hạng I, Điều 8 hạng II, Điều 9 hạng III), mỗi Điều có điểm c về truyền thông giáo dục sức khỏe; câu hỏi không nêu hạng). Đã nêu hạng II; id cũ vilextime:T1:provision:0fdffb50-2d40-11f1-ad9b-6dee35851177:2025-12-19: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>41/2025/TT-BYT · hiệu lực 2025-12-18 → nay · lúc thu thập: Còn hiệu lực
+Điều 8. Bác sĩ y học dự phòng chính (hạng II) - Mã số: V.08.02.05
+1. Nhiệm vụ:
+a) Tổ chức thực hiện nhiệm vụ phòng bệnh, cụ thể:
+- Xây dựng kế hoạch tổ chức thực hiện các hoạt động chuyên môn về phòng bệnh, quản lý chương trình y tế, truyền thông giáo dục sức khỏe, sức khỏe lao động, bệnh nghề nghiệp, tai nạn thương tích;
+- Tổ chức thực hiện hoạt động phòng, chống các bệnh truyền nhiễm: giám sát, phát hiện dịch bệnh, tiêm chủng phòng bệnh, kiểm soát, xử lý và khống chế dịch, bệnh, các tác nhân truyền nhiễm gây dịch nhất là dịch bệnh mới phát sinh;
+- Tổ chức thực hiện hoạt động phòng, chống các bệnh không lây nhiễm: phòng chống các yếu tố nguy cơ; sàng lọc, phát hiện sớm, quản lý, theo dõi người mắc bệnh không lây nhiễm, bệnh mạn tính;
+- Tổ chức triển khai thực hiện việc đánh giá tình trạng sức khỏe, các yếu tố nguy cơ và nhu cầu chăm sóc sức khỏe của cộng đồng;
+- Tổ chức thực hiện các hoạt động sức khỏe môi trường, sức khỏe nghề nghiệp: bảo đảm chất lượng nước sinh hoạt, phòng chống bệnh nghề nghiệp và phòng chống tai nạn, thương tích, quản lý chất thải y tế.
+b) Thực hiện việc khám bệnh, chữa bệnh cấp ban đầu, xử lý cấp cứu, khắc phục hậu quả thiên tai, thảm họa liên quan đến sức khỏe con người theo phạm vi hoạt động chuyên môn được giao;
+c) Tổ chức biên soạn nội dung và lập kế hoạch hướng dẫn công tác thông tin, giáo dục, truyền thông về bảo vệ, chăm sóc và nâng cao sức khỏe; đưa ra các biện pháp quản lý sức khỏe tại cộng đồng;
+d) Tổ chức triển khai các nội dung chăm sóc sức khỏe ban đầu;
+đ) Tham gia phân tích, đánh giá, kết luận những vấn đề chuyên môn về phòng bệnh khi có yêu cầu;
+e) Đào tạo và nghiên cứu khoa học:
+- Tổ chức biên soạn chương trình, tài liệu chuyên môn; xây dựng quy chế, quy trình kỹ thuật chuyên môn phòng bệnh; các giải pháp nhằm nâng cao chất lượng công tác phòng bệnh;
+- Tổ chức đào tạo, bồi dưỡng về lĩnh vực phòng bệnh phù hợp với trình độ và phạm vi chuyên môn đối với viên chức, người học;
+- Chủ trì hoặc tham gia các đề tài, chương trình, dự án nghiên cứu khoa học cấp Nhà nước, cấp bộ, cấp tỉnh;
+- Chủ trì hoặc tham gia nghiên cứu, cung cấp bằng chứng xây dựng chính sách, kế hoạch phát triển về công tác phòng bệnh của ngành, lĩnh vực, địa phương.</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -823,9 +882,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=0ae72df0-4247-11f1-9aef-8b444472143a</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -836,18 +892,40 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Hành vi sử dụng biển hiệu sai mẫu hoặc sai nội dung đăng ký hoạt động trong lĩnh vực bổ trợ tư pháp được xác định ra sao về mức xử phạt?»; nhãn cũ khong_dat question_ambiguous: 'Biển hiệu sai mẫu/sai nội dung trong lĩnh vực bổ trợ tư pháp' có ở Điều 9 (tổ chức hành nghề luật sư), 11 (tư vấn pháp luật), 17 (công chứng), 69 (thừa phát lại) với mức phạt khác nhau; câu hỏi không nêu nghề). Hỏi khung phạt tiền của hành vi trong lĩnh vực công chứng: 3–7 triệu theo câu dẫn; tổ chức gấp 02 lần theo khoản 4 Điều 4 NĐ 109/2026</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>109/2026/NĐ-CP · hiệu lực 2026-05-18 → nay · lúc thu thập: Còn hiệu lực
+Điều 17. Hành vi vi phạm quy định về hoạt động của tổ chức hành nghề công chứng
+1. Phạt tiền từ 3.000.000 đồng đến 7.000.000 đồng đối với một trong các hành vi sau:
+a) Không niêm yết hoặc niêm yết không đầy đủ lịch làm việc; thủ tục công chứng; nội quy tiếp người yêu cầu công chứng; phí công chứng, phí, giá dịch vụ theo yêu cầu liên quan đến việc công chứng và chi phí khác tại trụ sở của tổ chức mình;
+b) Đăng báo nội dung đăng ký hoạt động không đúng thời hạn hoặc không đầy đủ nội dung hoặc không đúng số lần theo quy định;
+c) Thực hiện không đúng hoặc không đầy đủ chế độ báo cáo; báo cáo không chính xác về tình hình tổ chức và hoạt động của tổ chức hành nghề công chứng;
+d) Lập, quản lý, sử dụng sổ hoặc sử dụng biểu mẫu trong hoạt động công chứng không đúng quy định;
+đ) Lưu trữ hồ sơ công chứng không đúng quy định;
+e) Sử dụng biển hiệu không đúng mẫu hoặc nội dung biển hiệu không đúng giấy đăng ký hoạt động;
+g) Phân công công chứng viên hướng dẫn tập sự không đúng quy định;
+h) Từ chối tiếp nhận người tập sự hành nghề công chứng do Sở Tư pháp chỉ định mà không có lý do chính đáng;
+i) Từ chối nhận lưu giữ di chúc mà không có lý do chính đáng hoặc từ chối tiếp nhận yêu cầu công bố di chúc khi có yêu cầu hợp lệ từ người thừa kế;
+k) Không duy trì việc đáp ứng điều kiện về trụ sở của tổ chức hành nghề công chứng theo quy định;
+l) Không ghi số văn bản công chứng hoặc không đóng dấu của tổ chức hành nghề công chứng vào văn bản công chứng đã có chữ ký của công chứng viên hoặc không đóng dấu giáp lai giữa các tờ đối với văn bản công chứng có từ 02 tờ trở lên hoặc không giao bản gốc văn bản công chứng cho người yêu cầu công chứng;
+m) Không mua bảo hiểm trách nhiệm nghề nghiệp liên tục cho công chứng viên của tổ chức mình;
+n) Không tạo điều kiện cho công chứng viên của tổ chức mình tham gia bồi dưỡng nghiệp vụ công chứng hằng năm;
+o) Không đề nghị cấp lại thẻ công chứng viên cho công chứng viên trong trường hợp tổ chức hành nghề công chứng thay đổi tên gọi;
+p) Vi phạm quy định về thông báo và gửi bản sao hợp đồng bảo hiểm, hợp đồng thay đổi, gia hạn hợp đồng bảo hiểm trách nhiệm nghề nghiệp của công chứng viên cho Sở Tư pháp khi mua bảo hiểm hoặc thay đổi, gia hạn hợp đồng bảo hiểm;
+q) Không phân công công chứng viên của tổ chức mình thực hiện việc công bố di chúc hoặc phân công trong trường hợp người lập di chúc đã chỉ định công chứng viên khác hiện đang hành nghề tại tổ chức hành nghề công chứng đó là người công bố di chúc;
+r) Không xác nhận và đóng dấu của tổ chức hành nghề công chứng vào bản sao di chúc về việc sao từ hồ sơ gửi giữ di chúc.</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -900,9 +978,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32779</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -913,7 +988,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
           <t>valid_to_wrong</t>
@@ -924,11 +998,24 @@
           <t>NĐ 176/2013/NĐ-CP đã bị NĐ 117/2020/NĐ-CP thay thế (hiệu lực 15/11/2020), valid_to vẫn rỗng · Mức trong đáp án là mức cho cá nhân; nếu người sử dụng lao động là tổ chức thì gấp 02 lần (khoản 5 quy định chung NĐ 176/2013); id cũ vilextime:T1:provision:2f5ea3c0-2c85-11f1-b760-79130d885196:2014-01-01: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>176/2013/NĐ-CP · hiệu lực 2013-12-31 → nay · lúc thu thập: Còn hiệu lực
+Điều 57. Vi phạm quy định về đóng bảo hiểm y tế
+3. Phạt tiền đối với hành vi không đóng bảo hiểm y tế cho toàn bộ số người lao động có trách nhiệm tham gia bảo hiểm y tế của người sử dụng lao động theo một trong các mức sau đây:
+a) Từ 500.000 đồng đến 1.000.000 đồng, khi vi phạm dưới 10 người lao động;
+b) Từ 1.000.000 đồng đến 5.000.000 đồng, khi vi phạm từ 10 đến dưới 50 người lao động;
+c) Từ 5.000.000 đồng đến 10.000.000 đồng, khi vi phạm từ 50 đến dưới 100 người lao động;
+d) Từ 10.000.000 đồng đến 15.000.000 đồng, khi vi phạm từ 100 đến dưới 500 người lao động;
+đ) Từ 15.000.000 đồng đến 20.000.000 đồng, khi vi phạm từ 500 đến dưới 1.000 người lao động;
+e) Từ 20.000.000 đồng đến 30.000.000 đồng, khi vi phạm từ 1.000 người lao động trở lên.</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -981,9 +1068,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=16750</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -994,18 +1078,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:312d0ee8-eb81-11f0-be34-83d33c77be02#k3:2006-04-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>61/2005/QH11 · hiệu lực 2006-04-01 → 2014-07-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 20. Chỉ định thầu
+3. Trước khi thực hiện chỉ định thầu quy định tại các điểm b, c, d và đ khoản 1 Điều này, dự toán đối với gói thầu đó phải được phê duyệt theo quy định.</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1058,9 +1147,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=32730</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1071,18 +1157,24 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:38528280-2c85-11f1-954b-d3e284a740f5:2014-02-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>206/2013/NĐ-CP · hiệu lực 2014-02-01 → 2026-01-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 21. Quyền, trách nhiệm của Bộ Tài chính
+1. Chủ trì nghiên cứu, xây dựng để báo cáo Chính phủ cơ chế về quản lý nợ của doanh nghiệp; hướng dẫn về các chỉ tiêu giám sát, đánh giá khả năng thanh toán nợ của doanh nghiệp; hướng dẫn chế độ trích lập và sử dụng các khoản dự phòng nợ phải thu khó đòi.
+Phối hợp tham gia với Bộ quản lý ngành, Ủy ban nhân dân cấp tỉnh trong việc giám sát, kiểm tra, đánh giá các khoản nợ của tập đoàn kinh tế nhà nước, tổng công ty nhà nước, công ty trách nhiệm hữu hạn một thành viên do Bộ quản lý ngành, Ủy ban nhân dân cấp tỉnh quyết định thành lập hoặc được giao quản lý.</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1135,9 +1227,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=46601</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1148,7 +1237,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -1159,11 +1247,17 @@
           <t>Citation 'Điểm b Khoản 2' thiếu phần/mục cha (path 'Chương I › Khoản 2'); id cũ vilextime:T1:provision:3c58dda6-e177-11f0-aad8-510bc3ddb5e6:2007-08-31: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>07/2007/TTLT-BTM-BTC · hiệu lực 2007-08-30 → 2019-11-05 · lúc thu thập: Hết hiệu lực toàn bộ
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1216,8 +1310,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=138874</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>document_ended 2024-07-15 bao_dong_gia</t>
@@ -1233,7 +1325,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
           <t>valid_to_wrong</t>
@@ -1244,11 +1335,28 @@
           <t>Có cạnh 'Văn bản được thay thế' trỏ vào TT 15/2019/TT-BNNPTNT nhưng valid_to rỗng; id cũ vilextime:T1:provision:45d941c0-2c83-11f1-a5f8-7129425f1ab5:2020-01-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>15/2019/TT-BNNPTNT · hiệu lực 2020-01-01 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 5. Dự toán
+1. Chi phí xây dựng:
+a) Chi phí trực tiếp, gồm:
+Chi phí nhân công: chuẩn bị hiện trường, trồng, chăm sóc, kiểm tra, giám sát, bảo vệ rừng và chi phí khác có liên quan;
+Chi phí máy và thiết bị thi công: làm đất, vận chuyển cây con bằng máy; san, ủi mặt bằng, làm đường ranh cản lửa và chi phí khác có liên quan;
+Chi phí vật tư: giống, phân bón, thuốc bảo vệ thực vật và các vật tư khác có liên quan.
+b) Chi phí chung: được tính bằng 5,0% chi phí trực tiếp, gồm:
+Chi phí trang bị bảo hộ, an toàn lao động và bảo vệ môi trường cho người lao động và môi trường xung quanh;
+Chi phí vận chuyển máy móc, thiết bị thi công và lực lượng lao động đến và ra khỏi công trường;
+Chi phí bảo đảm an toàn giao thông phục vụ thi công (nếu có).
+c) Thu nhập chịu thuế tính trước: là lợi nhuận dự tính trong dự toán xây dựng công trình, được tính bằng 5,5% tổng chi phí trực tiếp và chi phí chung;
+d) Thuế giá trị gia tăng thực hiện theo quy định của nhà nước.</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1301,9 +1409,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=185823</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1314,18 +1419,29 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:46db5bf0-31c7-11f1-ac1e-d38b84040a86:2026-02-16: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>341/2025/NĐ-CP · hiệu lực 2026-02-15 → nay · lúc thu thập: Còn hiệu lực
+Điều 36. Hành vi vận chuyển, tàng trữ hàng hóa sao chép lậu
+1. Phạt tiền đối với hành vi vận chuyển hàng hóa sao chép lậu theo quy định như sau:
+a) Từ 1.000.000 đồng đến 3.000.000 đồng trong trường hợp số lợi bất hợp pháp thu được dưới 10.000.000 đồng hoặc gây thiệt hại cho chủ sở hữu quyền tác giả, chủ sở hữu quyền liên quan dưới 20.000.000 đồng hoặc hàng hóa vi phạm trị giá dưới 20.000.000 đồng;
+b) Từ 3.000.000 đồng đến 5.000.000 đồng trong trường hợp số lợi bất hợp pháp thu được từ 10.000.000 đồng đến dưới 20.000.000 đồng hoặc gây thiệt hại cho chủ sở hữu quyền tác giả, chủ sở hữu quyền liên quan từ 20.000.000 đồng đến dưới 40.000.000 đồng hoặc hàng hóa vi phạm trị giá từ 20.000.000 đồng đến dưới 40.000.000 đồng;
+c) Từ 5.000.000 đồng đến 10.000.000 đồng trong trường hợp số lợi bất hợp pháp thu được từ 20.000.000 đồng đến dưới 30.000.000 đồng hoặc gây thiệt hại cho chủ sở hữu quyền tác giả, chủ sở hữu quyền liên quan từ 40.000.000 đồng đến dưới 60.000.000 đồng hoặc hàng hóa vi phạm trị giá từ 40.000.000 đồng đến dưới 60.000.000 đồng;
+d) Từ 10.000.000 đồng đến 20.000.000 đồng trong trường hợp số lợi bất hợp pháp thu được từ 30.000.000 đồng đến dưới 50.000.000 đồng hoặc gây thiệt hại cho chủ sở hữu quyền tác giả, chủ sở hữu quyền liên quan từ 60.000.000 đồng đến dưới 100.000.000 đồng hoặc hàng hóa vi phạm trị giá từ 60.000.000 đồng đến dưới 100.000.000 đồng;
+đ) Từ 20.000.000 đồng đến 30.000.000 đồng trong trường hợp số lợi bất hợp pháp thu được từ 50.000.000 đồng đến dưới 100.000.000 đồng hoặc gây thiệt hại cho chủ sở hữu quyền tác giả, chủ sở hữu quyền liên quan từ 100.000.000 đồng đến dưới 150.000.000 đồng hoặc hàng hóa vi phạm trị giá từ 100.000.000 đồng đến dưới 150.000.000 đồng;
+e) Từ 30.000.000 đồng đến 50.000.000 đồng trong trường hợp số lợi bất hợp pháp thu được từ 100.000.000 đồng trở lên hoặc gây thiệt hại cho chủ sở hữu quyền tác giả, chủ sở hữu quyền liên quan từ 150.000.000 đồng trở lên hoặc hàng hóa vi phạm trị giá từ 150.000.000 đồng trở lên.</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1378,9 +1494,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=18448</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1391,18 +1504,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Một người bị xử phạt vi phạm hành chính không tự nguyện nộp tiền phạt thì có thể bị áp dụng biện pháp cưỡng chế nào đối với tài sản của mình?»; nhãn cũ khong_dat question_ambiguous: Hỏi biện pháp cưỡng chế 'đối với tài sản'; khoản 1 (khấu trừ tiền từ tài khoản ngân hàng) cũng là biện pháp đối với tài sản). Câu hỏi chốt biện pháp dẫn tới bán đấu giá, chỉ khớp khoản 2; id cũ vilextime:T1:provision:4a1d663e-eb7f-11f0-a965-3115c99302b6#k2:2005-04-09: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>37/2005/NĐ-CP · hiệu lực 2005-04-08 → 2013-12-28 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 2. Các biện pháp cưỡng chế hành chính
+2. Kê biên phần tài sản có giá trị tương ứng với số tiền phạt để bán đấu giá;</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1430,7 +1548,6 @@
           <t>2010-08-12 (giua_khoang); 2026-05-02 (sau_het_hieu_luc)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>1. Vật chứng, ảảnh hoặc biên bản xác nhận vật chứng được đưa ra để xem xét tại phiên tòa.</t>
@@ -1451,9 +1568,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=19411</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1464,7 +1578,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -1475,11 +1588,18 @@
           <t>Chấm lại 28/09 trên câu hỏi đã sửa. Câu hỏi nay hỏi đúng việc xem xét vật chứng. Nút không có Điều cha trong cây nên citation "Điều 94" không kiểm được (theo trí nhớ thuộc Điều 212 BLTTHS 2003 — cần kiểm); id cũ vilextime:T1:provision:5003ac4e-eb7e-11f0-a0a3-c9aae40c2eb7:2004-07-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>19/2003/QH11 · hiệu lực 2004-07-01 → 2018-01-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 94. Huỷ bỏ hoặc thay thế biện pháp ngăn chặn
+1. Khi vụ án bị đình chỉ thì mọi biện pháp ngăn chặn đã áp dụng đều phải được huỷ bỏ.</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1532,9 +1652,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=19605</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1545,7 +1662,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -1556,11 +1672,17 @@
           <t>Citation chỉ còn 'Điểm a', path 'Phần 1 › Chương › Mục › Điểm a' mất số hiệu; id cũ vilextime:T1:provision:514503be-eb6f-11f0-8d3d-79ec914317f6:2004-02-21: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>01/2004/TT-BKH · hiệu lực 2004-02-20 → nay · lúc thu thập: Còn hiệu lực
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1613,9 +1735,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=176677</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1626,18 +1745,27 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:578ff710-29b8-11f1-b193-61b18a6e6e8f:2025-04-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>76/2025/NĐ-CP · hiệu lực 2025-04-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 5. Trình tự rà soát, hoàn thiện thủ tục, điều kiện được tiếp tục sử dụng đất, xác định lại giá đất, thu tiền sử dụng đất, tiền thuê đất đối với 13 dự án tại thành phố Đà Nẵng quy định tại Điều 4 Nghị quyết số 170/2024/QH15
+2. Trình tự rà soát điều kiện được tiếp tục sử dụng đất để thực hiện dự án được thực hiện như sau:
+a) Sở Nông nghiệp và Môi trường chủ trì, phối hợp với các cơ quan có liên quan rà soát các điều kiện quy định tại điểm a khoản 1 và điểm a khoản 2 Điều 4 Nghị quyết số 170/2024/QH15 đối với từng dự án về: sự phù hợp với quy hoạch sử dụng đất hoặc quy hoạch đô thị (quy hoạch chung hoặc quy hoạch phân khu) đã được phê duyệt theo quy định của pháp luật; không vi phạm quy hoạch sử dụng đất quốc phòng, quy hoạch sử dụng đất an ninh, quy hoạch 03 loại rừng (hoặc quy hoạch lâm nghiệp) đã được phê duyệt, điều kiện năng lực thực hiện dự án của nhà đầu tư;
+b) Sở Nông nghiệp và Môi trường tổng hợp kết quả đánh giá điều kiện và lập hồ sơ trình Ủy ban nhân dân thành phố Đà Nẵng xem xét, đánh giá điều kiện đối với từng dự án được tiếp tục sử dụng đất; hồ sơ gồm tờ trình, dự thảo quyết định đánh giá dự án đủ điều kiện được tiếp tục sử dụng đất, ý kiến của các cơ quan liên quan;
+c) Trong thời hạn không quá 05 ngày làm việc kể từ ngày nhận được hồ sơ do Sở Nông nghiệp và Môi trường trình, Ủy ban nhân dân thành phố Đà Nẵng xem xét về các điều kiện và ban hành quyết định đánh giá dự án đủ điều kiện được tiếp tục sử dụng đất gửi Sở Nông nghiệp và Môi trường;
+d) Thời gian hoàn thành các công việc quy định tại khoản này chậm nhất là 06 tháng kể từ ngày Ủy ban nhân dân thành phố Đà Nẵng ban hành quyết định được tiếp tục thực hiện rà soát các điều kiện theo quy định tại điểm d khoản 1 Điều này.</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1690,9 +1818,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=172311</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1703,18 +1828,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:596e6fe0-2c7d-11f1-b48b-4383f69de024:2025-01-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>68/2024/TT-BQP · hiệu lực 2025-01-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 3. Giải thích từ ngữ
+5. Cơ sở đào tạo lái xe quân sự là các cơ sở đào tạo thuộc phạm vi quản lý của Bộ Quốc phòng có chức năng đào tạo lái xe quân sự.</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1767,9 +1897,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=163057</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1780,18 +1907,27 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:5ad876ec-eb72-11f0-9841-0f234bceec4b:2023-09-16: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>32/2023/TT-BCA · hiệu lực 2023-09-15 → 2025-01-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 20. Xử lý vi phạm trong khi tuần tra, kiểm soát
+2. Xử phạt vi phạm hành chính có lập biên bản
+a) Khi phát hiện vi phạm hành chính thuộc trường hợp xử phạt vi phạm hành chính có lập biên bản, cán bộ Cảnh sát giao thông thực hiện lập biên bản vi phạm hành chính theo quy định. Biên bản vi phạm hành chính được lập bằng mẫu in sẵn hoặc lập trên Hệ thống cơ sở dữ liệu xử lý vi phạm hành chính;
+b) Khi lập xong biên bản vi phạm hành chính, cán bộ lập biên bản đọc lại cho những người có tên trong biên bản cùng nghe; hướng dẫn quyền, thời hạn giải trình về vi phạm hành chính đối với hành vi vi phạm hành chính mà cá nhân, tổ chức có quyền giải trình theo quy định tại Điều 61 Luật Xử lý vi phạm hành chính (sửa đổi, bổ sung năm 2020); đề nghị người vi phạm cung cấp số điện thoại liên hệ (nếu có) để nhận thông tin xử phạt thông qua Cổng dịch vụ công Quốc gia, Cổng dịch vụ công Bộ Công an; ký vào biên bản (trường hợp người vi phạm không ký được thì điểm chỉ), trừ trường hợp biên bản được lập theo quy định tại khoản 7 Điều 58 Luật Xử lý vi phạm hành chính (sửa đổi, bổ sung năm 2020). Trường hợp có người chứng kiến, người phiên dịch, người bị thiệt hại hoặc đại diện tổ chức bị thiệt hại thì những người này cùng phải ký vào biên bản; biên bản vi phạm hành chính gồm nhiều trang, thì phải ký vào từng trang biên bản;
+c) Trường hợp người vi phạm không có mặt tại nơi vi phạm hoặc cố tình trốn tránh hoặc vì lý do khách quan mà không ký, điểm chỉ vào biên bản hoặc có mặt nhưng từ chối ký, điểm chỉ vào biên bản hoặc trường hợp không xác định được đối tượng vi phạm thì Tổ trưởng Tổ Cảnh sát giao thông mời đại diện chính quyền cấp xã nơi xảy ra vi phạm hoặc ít nhất 01 người chứng kiến ký vào biên bản xác nhận việc người vi phạm không ký, điểm chỉ vào biên bản; trường hợp không có chữ ký của đại diện chính quyền cấp xã hoặc của người chứng kiến thì cán bộ Cảnh sát giao thông phải ghi rõ lý do vào biên bản. Sử dụng phương tiện, thiết bị kỹ thuật nghiệp vụ ghi nhận vụ việc và phải báo cáo thủ trưởng đơn vị bằng văn bản để làm cơ sở cho người có thẩm quyền xem xét, quyết định xử phạt;
+d) Việc giao biên bản vi phạm hành chính cho người vi phạm thực hiện theo quy định tại Điều 58 Luật Xử lý vi phạm hành chính (sửa đổi, bổ sung năm 2020) và Điều 12 Nghị định số 118/2021/NĐ-CP ngày 23/12/2021 của Chính phủ quy định chi tiết một số điều và biện pháp thi hành Luật Xử lý vi phạm hành chính (sau đây viết gọn là Nghị định số 118/2021/NĐ-CP).</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1844,9 +1980,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=6776a0a0-543a-11f1-9456-0b6fbb8f8274</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1857,7 +1990,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr">
         <is>
           <t>citation_path_wrong,group_wrong</t>
@@ -1868,11 +2000,17 @@
           <t>Đơn vị là lời văn trích trong thông tư sửa đổi 121/2025/TT-BTC; citation thiếu Điều ('Điểm b Khoản 2'); thực chất là phiên bản mới của điều khoản thuộc thông tư bị sửa; id cũ vilextime:T1:provision:5e8c584c-543d-11f1-ae49-0120c8b0e422:2026-02-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>121/2025/TT-BTC · hiệu lực 2026-02-01 → nay · lúc thu thập: Hết hiệu lực một phần
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1925,9 +2063,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=30386</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -1938,7 +2073,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr">
         <is>
           <t>valid_to_wrong</t>
@@ -1949,11 +2083,23 @@
           <t>NĐ 24/2013/NĐ-CP đã bị NĐ 123/2015/NĐ-CP thay thế (hiệu lực 01/01/2016); valid_to vẫn rỗng; id cũ vilextime:T1:provision:5ed1beca-2c86-11f1-841a-7d89578d89e1:2013-05-16: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>24/2013/NĐ-CP · hiệu lực 2013-05-15 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 17. Thẩm quyền, trình tự, thủ tục ghi vào sổ đăng ký kết hôn việc kết hôn của công dân Việt Nam đã được giải quyết tại cơ quan có thẩm quyền của nước ngoài ở nước ngoài
+2. Hồ sơ ghi vào sổ việc kết hôn được lập thành 01 bộ, gồm các giấy tờ sau:
+a) Tờ khai ghi vào sổ việc kết hôn (theo mẫu quy định);
+b) Bản sao giấy tờ chứng nhận việc kết hôn do cơ quan có thẩm quyền của nước ngoài cấp;
+c) Bản sao một trong các giấy tờ để chứng minh về nhân thân, như Giấy chứng minh nhân dân, Hộ chiếu hoặc giấy tờ hợp lệ thay thế;
+d) Bản sao sổ hộ khẩu hoặc sổ tạm trú của người có yêu cầu.
+Trường hợp công nhận việc kết hôn giữa công dân Việt Nam với người nước ngoài mà trước đó công dân Việt Nam hoặc người nước ngoài đã ly hôn với công dân Việt Nam tại cơ quan có thẩm quyền của nước ngoài thì phải nộp Giấy xác nhận về việc ghi vào sổ hộ tịch việc ly hôn đã tiến hành ở nước ngoài theo quy định của pháp luật Việt Nam.</t>
+        </is>
+      </c>
+      <c r="Y19" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2006,9 +2152,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111050</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2019,18 +2162,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:624d3820-2dbe-11f1-ad11-45ab3867d967:2016-07-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>60/2016/NĐ-CP · hiệu lực 2016-07-01 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 25. Danh mục chế phẩm sinh học trong xử lý chất thải tại Việt Nam
+2. Định kỳ 06 tháng một lần, Tổng cục Môi trường có trách nhiệm rà soát, sửa đổi, bổ sung danh mục chế phẩm sinh học trong xử lý chất thải tại Việt Nam.</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2083,9 +2231,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=144776</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2096,18 +2241,25 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:67b6aac0-eada-11f0-9fe9-9f5f3d9c1c27#k16#b:2015-03-11: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>85/2014/TT-BGTVT · hiệu lực 2015-03-10 → 2025-01-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 4. Các quy định khi cải tạo xe cơ giới
+16. Khối lượng toàn bộ cho phép tham gia giao thông của xe cơ giới sau cải tạo phải đảm bảo:
+a) Đối với xe chở người: Không lớn hơn giá trị nhỏ của khối lượng toàn bộ theo thiết kế tương ứng với số người cho phép chở lớn nhất theo thiết kế của nhà sản xuất và khối lượng toàn bộ cho phép tham gia giao thông theo quy định về tải trọng cầu đường.
+b) Đối với xe tải và xe chuyên dùng: Không lớn hơn giá trị của khối lượng toàn bộ theo thiết kế của nhà sản xuất và khối lượng toàn bộ cho phép tham gia giao thông theo quy định về tải trọng cầu đường.</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2160,9 +2312,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=44169</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2173,7 +2322,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr">
         <is>
           <t>valid_to_wrong</t>
@@ -2184,11 +2332,18 @@
           <t>Luật Tổ chức TAND 62/2014/QH13 đã bị Luật Tổ chức TAND 34/2024/QH15 thay thế từ 01/01/2025; valid_to vẫn rỗng; id cũ vilextime:T1:provision:680053d0-2768-11f1-bfbd-efc08bd225d4:2015-06-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>62/2014/QH13 · hiệu lực 2015-06-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 78. Điều động Thẩm phán
+2. Chánh án Tòa án nhân dân tối cao quyết định điều động Thẩm phán từ Tòa án nhân dân này đến làm nhiệm vụ tại Tòa án nhân dân khác không cùng phạm vi thẩm quyền theo lãnh thổ hoặc không cùng một tỉnh, thành phố trực thuộc trung ương.</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2241,9 +2396,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=179711</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2254,18 +2406,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp cơ sở khám bệnh, chữa bệnh không có đơn giá làm căn cứ thanh toán, quỹ bảo hiểm y tế thanh toán theo đơn giá nào?»; nhãn cũ khong_dat question_ambiguous: Khoản 4, 5, 6 cùng là 'trường hợp không có đơn giá ...' theo tầng; câu hỏi không chỉ ra tầng nào). Câu hỏi nêu tầng 'tỉnh và tỉnh giáp ranh đều không có' (khoản 5) nên chỉ khớp khoản 6; id cũ vilextime:T1:provision:6836992a-2e86-11f1-b466-61cabd0bcac0:2025-08-16: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>188/2025/NĐ-CP · hiệu lực 2025-08-15 → nay · lúc thu thập: Còn hiệu lực
+Điều 49. Thanh toán chi phí mua thuốc, hóa chất, vật tư xét nghiệm, thiết bị y tế cho cơ sử khám bệnh, chữa bệnh là đơn vị sự nghiệp công lập tư bảo đảm chi thường xuyên và chi đầu tư, đơn vị sự nghiệp công lập tự bảo đảm chi thường xuyên và các cơ sở khám bệnh, chữa bệnh tư nhân thuộc trường hợp quy định tại khoản 3 Điều 55 của Luật Đấu thầu năm 2023 được sửa đổi, bổ sung bởi Luật số 90/2025/QH15
+6. Trường hợp không có đơn giá quy định tại khoản 5 Điều này, quỹ bảo hiểm y tế thanh toán theo đơn giá trúng thầu của cơ sở khám bệnh, chữa bệnh của Nhà nước, kết quả mua sắm tập trung trên địa bàn tỉnh khác trên toàn quốc theo nguyên tắc quy định tại các điểm a, b và c khoản 5 Điều này.</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2318,9 +2475,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=18116</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2331,18 +2485,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp các đơn vị thuộc Sở Tài chính cần thực hiện quy định pháp luật về thanh tra, Chánh Thanh tra Sở có nhiệm vụ gì đối với thủ trưởng các đơn vị đó?»; nhãn cũ khong_dat question_ambiguous: Khoản 6 cũng là nhiệm vụ của Chánh Thanh tra Sở đối với thủ trưởng đơn vị thuộc Sở về thực hiện pháp luật thanh tra). Câu hỏi chốt 'hướng dẫn, đôn đốc', khác khoản 6; id cũ vilextime:T1:provision:683af2ca-df3c-11f0-b581-0d9a21390744#k4:2005-07-19: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>81/2005/NĐ-CP · hiệu lực 2005-07-18 → 2012-11-25 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 15. Nhiệm vụ, quyền hạn của Chánh Thanh tra Sở
+4. H­ướng dẫn, đôn đốc Thủ tr­ưởng tổ chức, đơn vị thuộc quyền quản lý của Sở Tài chính thực hiện các quy định pháp luật về thanh tra.</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2395,9 +2554,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133210</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2408,18 +2564,26 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Pháp luật về quản lý an toàn trong hoạt động dầu khí quy định chương trình quản lý an toàn phải được thực hiện vào những thời điểm nào của công trình?»; nhãn cũ khong_dat question_ambiguous: Hỏi 'những thời điểm nào' nhưng đáp án chỉ là điểm a; điểm b, c cũng là thời điểm thực hiện). Câu hỏi chốt giai đoạn xây dựng, chỉ khớp điểm a; id cũ vilextime:T1:provision:69823b0a-df52-11f0-ac04-13973f36b963:2018-12-15: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>40/2018/TT-BCT · hiệu lực 2018-12-14 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 4. Thời điểm xây dựng các tài liệu quản lý an toàn
+1. Chương trình quản lý an toàn được thực hiện:
+a) Trước khi thi công, xây dựng, lắp đặt.
+b) Trước khi chạy thử, vận hành.
+c) Trước khi hoán cải, thay đổi công suất, công nghệ, thu dọn công trình khi kết thúc khai thác hoặc kết thúc dự án, thay đổi chính sách an toàn và hệ thống quản lý an toàn.</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2472,9 +2636,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=122988</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2485,18 +2646,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:77282ab0-3c74-11f1-b2ff-b7688e5b9a17:2018-01-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>15/2017/QH14 · hiệu lực 2018-01-01 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 126. Trách nhiệm xây dựng Hệ thống thông tin về tài sản công
+2. Bộ Tài chính có trách nhiệm tổ chức xây dựng, quản lý, vận hành, khai thác Hệ thống thông tin về tài sản công thuộc phạm vi quản lý.</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2549,9 +2715,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=18566</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2562,18 +2725,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:790c983e-eb89-11f0-bfbc-3b8923ed9a01#k3:2005-07-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>27/2004/QH11 · hiệu lực 2005-07-01 → 2019-07-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 69. Người giám định
+3. Người giám định từ chối kết luận giám định mà không có lý do chính đáng hoặc kết luận giám định sai sự thật hoặc khi được cơ quan trưng cầu giám định triệu tập mà vắng mặt không có lý do chính đáng thì phải chịu trách nhiệm theo quy định của pháp luật.</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2626,9 +2794,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=19465</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2639,18 +2804,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:7955ccf0-335c-11f1-85de-b1296396b4f2:2004-09-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>17/2004/PL-UBTVQH11 · hiệu lực 2004-09-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 2. Phạm vi điều chỉnh
+Pháp lệnh này quy định việc xây dựng, tổ chức quản lý, điều hành và sử dụng dự trữ quốc gia.</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2703,9 +2873,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=146471</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2716,18 +2883,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:79b8bd90-227e-11f1-8c2a-e9c4dd423d40:2021-02-06: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>147/2020/NĐ-CP · hiệu lực 2021-02-05 → nay · lúc thu thập: Còn hiệu lực
+Điều 38. Vốn nhận ủy thác
+Vốn nhận ủy thác theo quy định tại Điều 32 Nghị định này không thuộc vốn hoạt động của Quỹ đầu tư phát triển địa phương và được hạch toán, quản lý tách bạch với vốn hoạt động của Quỹ.</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2780,9 +2952,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=37527</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2793,7 +2962,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr">
         <is>
           <t>valid_to_wrong</t>
@@ -2804,11 +2972,20 @@
           <t>Có cạnh 'Văn bản được thay thế' trỏ vào TT 147/2014/TT-BTC nhưng valid_to rỗng; id cũ vilextime:T1:provision:886734ba-eae9-11f0-bfb6-1b525bfe6ee3:2014-11-26: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>147/2014/TT-BTC · hiệu lực 2014-11-25 → nay · lúc thu thập: Còn hiệu lực
+Điều 13. Thu nhập của Quỹ bảo lãnh tín dụng
+2. Thu về hoạt động tài chính:
+a) Thu lãi tiền gửi tại Kho bạc Nhà nước, ngân hàng thương mại nơi Quỹ bảo lãnh tín dụng mở tài khoản;
+b) Thu lãi đầu tư trái phiếu Chính phủ.</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2861,9 +3038,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=14704</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2874,7 +3048,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -2885,11 +3058,17 @@
           <t>Citation 'Điểm d Khoản 2' thiếu Phần/Mục (path 'Phần › Chương › Khoản 2'); id cũ vilextime:T1:provision:89b5eb36-df3b-11f0-be0a-a597416047b7:2007-02-15: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>03/2007/NQ-CP · hiệu lực 2007-02-14 → nay · lúc thu thập: Còn hiệu lực
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2942,9 +3121,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=111829</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -2955,18 +3131,25 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:89f4e824-df4d-11f0-947a-55d04134c924#k2#b:2016-01-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>70/2015/TT-BGTVT · hiệu lực 2016-01-01 → 2021-10-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 1. Phạm vi điều chỉnh
+2. Thông tư này không áp dụng đối với:
+a) Xe mô tô, xe gắn máy, máy kéo và các loại xe tương tự;
+b) Xe cơ giới của quân đội, công an sử dụng vào mục đích quốc phòng, an ninh.</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3019,9 +3202,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=113098</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3032,18 +3212,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:8b621ba6-df47-11f0-8be7-01dbfc483b14#k4:2015-12-06: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
+          <t>97/2015/NĐ-CP · hiệu lực 2015-12-05 → 2020-12-31 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 17. Tiêu chí đánh giá không hoàn thành nhiệm vụ
+4. Vi phạm điều lệ, nội quy, quy chế của tập đoàn, tổng công ty, công ty;</t>
+        </is>
+      </c>
+      <c r="Y33" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3096,8 +3281,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=119515</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>missed_event 2023-03-01 bao_dong_gia</t>
@@ -3113,18 +3296,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Pháp luật về chế độ làm việc của nhà giáo giáo dục nghề nghiệp quy định cách tính tiền lương dạy thêm giờ như thế nào?»; nhãn cũ khong_dat unanswerable_as_asked: Đáp án chỉ dẫn chiếu 'theo quy định hiện hành', không nêu cách tính mà câu hỏi hỏi). Câu hỏi hỏi căn cứ tính; đáp án chỉ dẫn chiếu quy định hiện hành nhưng trả lời đúng điều được hỏi; id cũ vilextime:T1:provision:8be75e80-2d47-11f1-bbcc-93110808d881:2017-07-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
+          <t>07/2017/TT-BLĐTBXH · hiệu lực 2017-07-01 → 2026-02-12 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 9. Chế độ dạy thêm giờ
+4. Cách tính trả lương dạy thêm giờ theo quy định hiện hành.</t>
+        </is>
+      </c>
+      <c r="Y34" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3177,9 +3365,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=15828</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3190,18 +3375,29 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:943871ea-df50-11f0-9561-3d5192b5741d:2006-10-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
-      <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
+      <c r="X35" s="2" t="inlineStr">
+        <is>
+          <t>66/2006/QH11 · hiệu lực 2006-10-01 → 2010-08-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 4.
+3. Cơ quan thẩm tra tiến hành thẩm tra những nội dung chủ yếu sau đây:
+a) Sự cần thiết đầu tư;
+b) Sự phù hợp với quy hoạch phát triển kinh tế - xã hội, quy hoạch phát triển ngành, lĩnh vực; quy hoạch sử dụng đất, tài nguyên; phương án di dân, tái định canh, định cư;
+c) Việc tuân thủ các quy định của pháp luật;
+d) Sự đáp ứng tiêu chí xác định dự án, công trình là dự án, công trình quan trọng quốc gia;
+đ) Những thông số cơ bản của dự án, công trình bao gồm: quy mô; hình thức đầu tư; địa điểm; diện tích đất cần sử dụng; thời gian, tiến độ thực hiện; phương án lựa chọn công nghệ; giải pháp bảo vệ môi trường; nguồn vốn, khả năng thu hồi vốn và trả nợ vốn vay;
+e) Hiệu quả kinh tế - xã hội ở mức báo cáo tiền khả thi.</t>
+        </is>
+      </c>
+      <c r="Y35" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3254,9 +3450,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=49828ac0-6e5a-11f1-b670-d3ec94724b75</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3267,7 +3460,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -3278,11 +3470,17 @@
           <t>Citation 'Điểm c Khoản 5' thiếu Điều (path 'Chương V › Mục 2 › Khoản 5'); id cũ vilextime:T1:provision:9e092383-44c5-47d8-94fe-4379606bf0ec:2026-07-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr"/>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>205/2026/NĐ-CP · hiệu lực 2026-07-01 → nay · lúc thu thập: Còn hiệu lực
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y36" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3335,9 +3533,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=27889</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3348,7 +3543,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -3359,11 +3553,41 @@
           <t>Mục 4.1 bị ghi thành 'Điểm 4 Khoản 4 Điều 4'</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
+      <c r="X37" s="2" t="inlineStr">
+        <is>
+          <t>188/2012/TT-BTC · hiệu lực 2012-12-28 → nay · lúc thu thập: Còn hiệu lực
+Điều 4. Hồ sơ, thủ tục hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất
+4. Quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất:
+4.1. Chậm nhất trong vòng 90 ngày kể từ ngày kết thúc năm tài chính, các ngân hàng thương mại nhà nước phải gửi hồ sơ đề nghị quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất cho Bộ Tài chính. Đối với các trường hợp hồ sơ không hợp lệ, Bộ Tài chính có trách nhiệm thông báo bằng văn bản cho các ngân hàng thương mại nhà nước trong thời hạn 10 ngày.
+4.2. Hồ sơ đề nghị quyết toán:
+a) Hồ sơ đề nghị quyết toán đối với khoản vay được hỗ trợ lãi suất vay vốn:
+- Báo cáo tổng hợp toàn hệ thống về quyết toán hỗ trợ lãi suất vay vốn đã được kiểm toán bởi Kiểm toán độc lập hoặc Kiểm toán nhà nước (Biểu 1 đính kèm).
+- Báo cáo theo từng tỉnh về quyết toán hỗ trợ lãi suất vay vốn (Biểu 2 đính kèm).
+b) Hồ sơ đề nghị quyết toán đối với khoản vay được cấp bù chênh lệch lãi suất:
+- Báo cáo tổng hợp toàn hệ thống về quyết toán chênh lệch lãi suất cấp bù theo lãi suất tín dụng đầu tư phát triển đã được kiểm toán bởi Kiểm toán độc lập hoặc Kiểm toán nhà nước (Biểu 3 đính kèm).
+- Báo cáo theo từng tỉnh về quyết toán chênh lệch lãi suất cấp bù theo lãi suất tín dụng đầu tư phát triển (Biểu 4 đính kèm).
+4.3. Các ngân hàng thương mại nhà nước tổ chức sao, lưu chứng từ, các báo cáo chi tiết theo từng khoản hỗ trợ lãi suất đảm bảo tính chính xác, minh bạch rõ ràng để tạo điều kiện cho công tác thẩm tra số liệu quyết toán hỗ trợ lãi suất và cấp bù chênh lệch lãi suất quy định tại Điểm 4.4 Khoản 4 Điều này.
+4.4. Thẩm tra số liệu quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất:
+a) Bộ Tài chính tiến hành thẩm tra số liệu quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất sau khi nhận được đầy đủ hồ sơ đề nghị quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất.
+b) Bộ Tài chính thông báo bằng văn bản các chi nhánh của ngân hàng thương mại nhà nước được lựa chọn để thực hiện thẩm tra quyết toán.
+c) Các ngân hàng thương mại nhà nước có trách nhiệm cung cấp các hồ sơ chi tiết theo từng khoản vay, được tổng hợp theo từng chi nhánh được lựa chọn để thực hiện thẩm tra quyết toán như sau:
+- Hợp đồng tín dụng, khế ước hoặc các giấy tờ tương đương để xác định đối tượng khách hàng vay vốn, tình hình thực hiện cho vay, dư nợ, thu nợ.
+- Bảng kê tích số để xác định số tiền hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất.
+- Giấy xác nhận của khách hàng trực tiếp đi vay vốn về việc đã được hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất theo năm trong đó có liệt kê từng lần được hỗ trợ dưới mọi hình thức.
+Các tài liệu nêu trên là bản phôtô có đóng dấu sao y bản chính của các ngân hàng thương mại nhà nước (số lượng 01 bộ) và được người có trách nhiệm ký, ghi rõ họ tên.
+d) Việc thẩm tra số liệu quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất được thực hiện trong thời gian 90 ngày kể từ ngày nhận được đầy đủ hồ sơ quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất của các ngân hàng thương mại nhà nước.
+4.5. Xử lý chênh lệch số liệu quyết toán và số tạm cấp hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất:
+- Trường hợp có sự chênh lệch giữa số báo cáo quyết toán có xác nhận của cơ quan kiểm toán và số thẩm tra quyết toán của Bộ Tài chính, các ngân hàng thương mại nhà nước có trách nhiệm điều chỉnh trên sổ sách kế toán để phản ánh chính xác số quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất.
+- Trường hợp số tạm cấp hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất đã được ngân sách nhà nước chuyển tiền cao hơn số thẩm tra quyết toán thì số chênh lệch sẽ được Bộ Tài chính thu hồi nộp ngân sách nhà nước.
+- Việc xử lý chênh lệch giữa số thẩm tra quyết toán và số tạm cấp hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất được thực hiện trong thời gian 45 ngày kể từ ngày của Biên bản thẩm tra quyết toán.
+- Trường hợp phải kéo dài thời gian xử lý chênh lệch giữa số liệu quyết toán và số thẩm tra quyết toán hỗ trợ lãi suất vay vốn và cấp bù chênh lệch lãi suất và các trường hợp đặc biệt khác sẽ do Bộ trưởng Bộ Tài chính xem xét, quyết định.</t>
+        </is>
+      </c>
+      <c r="Y37" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3416,9 +3640,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=129226</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3429,18 +3650,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:a7be8856-df43-11f0-bc93-d9f1eab2568f:2018-07-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>28/2018/TT-BGTVT · hiệu lực 2018-07-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 3. Giải thích từ ngữ
+1. Cung cấp thông tin hỗ trợ cảnh giới tại các điểm giao cắt giữa đường bộ, đường sắt là việc cung cấp thông tin của doanh nghiệp kinh doanh kết cấu hạ tầng đường sắt, chủ sở hữu đường sắt chuyên dùng thuộc phạm vi quản lý cho người cảnh giới để thực hiện nhiệm vụ tại vị trí cần cảnh giới.</t>
+        </is>
+      </c>
+      <c r="Y38" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3493,9 +3719,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=25420</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3506,18 +3729,27 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:a82e7fd0-2f43-11f1-845f-b378206c5594:2010-08-11: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>69/2010/NĐ-CP · hiệu lực 2010-08-10 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 12. Thẩm quyền, trình tự, thủ tục công nhận, thu hồi quyết định công nhận Phòng thí nghiệm nghiên cứu về sinh vật biến đổi gen
+2. Tổ chức đăng ký công nhận Phòng thí nghiệm nghiên cứu về sinh vật biến đổi gen phải nộp ba (03) bộ hồ sơ cho Bộ Khoa học và Công nghệ. Hồ sơ bao gồm:
+a) Đơn đăng ký công nhận Phòng thí nghiệm nghiên cứu về sinh vật biến đổi gen theo mẫu của Bộ Khoa học và Công nghệ;
+b) Bản sao các quyết định về chức năng, nhiệm vụ của tổ chức;
+c) Thuyết minh về năng lực của Phòng thí nghiệm nghiên cứu về sinh vật biến đổi gen theo mẫu của Bộ Khoa học và Công nghệ;
+d) Tài liệu liên quan chứng minh Phòng thí nghiệm nghiên cứu về sinh vật biến đổi gen đáp ứng các điều kiện quy định tại Điều 11 của Nghị định này.</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3570,9 +3802,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=23838</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3583,18 +3812,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:ac625f20-eadf-11f0-bd15-e99c4454aa60#k15:2009-12-23: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr"/>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr"/>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>134/2009/QĐ-TTg · hiệu lực 2009-12-22 → 2015-04-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 2. Nhiệm vụ và quyền hạn
+15. Thực hiện công tác cải cách hành chính theo mục tiêu và nội dung chương trình cải cách hành chính nhà nước đã được cấp có thẩm quyền phê duyệt.</t>
+        </is>
+      </c>
+      <c r="Y40" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3647,9 +3881,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=186231</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3660,18 +3891,25 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:ad505bc0-30b3-11f1-a005-81dac526b4c8:2026-02-17: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
-      <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>84/2025/TT-NHNN · hiệu lực 2026-02-16 → nay · lúc thu thập: Còn hiệu lực
+Điều 3. Giải thích từ ngữ
+3. Các đơn vị thuộc NHNN bao gồm: các đơn vị NHNN và các đơn vị sự nghiệp thuộc NHNN (không bao gồm các đơn vị trực tiếp nhận, quyết toán kinh phí với Ngân sách Nhà nước), cụ thể:
+a) Các đơn vị NHNN là các đơn vị kế toán phụ thuộc, bao gồm: NHNN Chi nhánh Khu vực; Vụ Tài chính - Kế toán; Sở Giao dịch; Văn phòng; Cục Quản lý ngoại hối; Cục Công nghệ thông tin; Cục Phát hành và Kho quỹ; Chi cục Công nghệ thông tin; Chi cục Phát hành và Kho quỹ; và các đơn vị NHNN có dự án hỗ trợ phát triển chính thức (dự án ODA);
+b) Các đơn vị sự nghiệp thuộc NHNN là các đơn vị kế toán độc lập, trực thuộc NHNN, bao gồm: Trung tâm thông tin tín dụng Quốc gia Việt Nam, Thời báo Ngân hàng, và Ban Quản lý dự án đầu tư xây dựng chuyên ngành.</t>
+        </is>
+      </c>
+      <c r="Y41" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3724,9 +3962,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=26151</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3737,18 +3972,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:b063dc28-e181-11f0-99cf-1f4f4f29cdc1#k2:2011-03-16: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr"/>
-      <c r="T42" t="inlineStr"/>
-      <c r="U42" t="inlineStr"/>
-      <c r="V42" t="inlineStr"/>
-      <c r="W42" t="inlineStr"/>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>01/2011/TT-BXD · hiệu lực 2011-03-15 → 2019-08-15 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 13. Nội dung ĐMC trong quy hoạch phân khu
+2. Đánh giá diễn biến môi trường khu vực, dự báo, so sánh các tác động môi trường của các phương án quy hoạch trên cơ sở mật độ xây dựng, quy hoạch sử dụng đất, bố trí các khu chức năng.</t>
+        </is>
+      </c>
+      <c r="Y42" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3801,9 +4041,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152647</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3814,18 +4051,30 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:b3bcbe30-21be-11f1-af12-01dc2ecd3981:2022-01-08: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr"/>
-      <c r="T43" t="inlineStr"/>
-      <c r="U43" t="inlineStr"/>
-      <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr"/>
+      <c r="X43" s="2" t="inlineStr">
+        <is>
+          <t>06/2022/NĐ-CP · hiệu lực 2022-01-07 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 29. Trách nhiệm trong quản lý các chất được kiểm soát
+1. Bộ Tài nguyên và Môi trường là cơ quan đầu mối quốc gia thực hiện Công ước Viên và Nghị định thư Montreal, chịu trách nhiệm trước Chính phủ thực hiện quản lý nhà nước về các chất được kiểm soát. Bộ Tài nguyên và Môi trường có trách nhiệm chủ trì, phối hợp với các bộ, ngành liên quan:
+a) Thực hiện quản lý các chất được kiểm soát theo điều ước quốc tế về bảo vệ tầng ô-dôn mà Việt Nam là thành viên; phân bổ, điều chỉnh, bổ sung hạn ngạch sản xuất, nhập khẩu các chất HCFC, HFC theo giai đoạn và hằng năm;
+b) Xây dựng, trình Thủ tướng Chính phủ ban hành Kế hoạch quốc gia về quản lý, loại trừ các chất được kiểm soát; trình cấp có thẩm quyền ban hành, sửa đổi, bổ sung danh mục, hướng dẫn sử dụng các chất được kiểm soát và quy định về điều kiện sản xuất, sử dụng các chất được kiểm soát theo cam kết thực hiện điều ước quốc tế về bảo vệ tầng ô-dôn mà nước Cộng hòa xã hội chủ nghĩa Việt Nam là thành viên;
+c) Công bố, sửa đổi, bổ sung danh mục các mặt hàng cấm xuất khẩu, cấm nhập khẩu; danh mục các mặt hàng được phép xuất khẩu, nhập khẩu theo điều kiện kèm theo mã số hàng hóa thuộc phạm vi quản lý trên cơ sở thống nhất với Bộ Công Thương về danh mục hàng hóa và thống nhất với Bộ Tài chính về mã số hàng hóa;
+d) Xây dựng và vận hành hệ thống dịch vụ công trực tuyến về đăng ký, báo cáo, phân bổ và quản lý hạn ngạch sản xuất, nhập khẩu các chất được kiểm soát; kết nối Cổng thông tin một cửa quốc gia về quản lý các chất được kiểm soát;
+đ) Tổ chức việc thực hiện các nghĩa vụ của quốc gia đối với Nghị định thư Montreal; phối hợp với cơ quan đầu mối của các quốc gia khác trong việc thực hiện các biện pháp tuân thủ Nghị định thư Montreal của Việt Nam;
+e) Thực hiện thanh tra, kiểm tra, giám sát việc đăng ký, báo cáo, sử dụng hạn ngạch; quản lý việc thu gom, tái sử dụng, tái chế và xử lý các chất được kiểm soát;
+g) Tổ chức thực hiện các nội dung được giao theo quy định của Luật Bảo vệ môi trường, Nghị định này và các nhiệm vụ khác liên quan đến quản lý chất được kiểm soát.</t>
+        </is>
+      </c>
+      <c r="Y43" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3878,9 +4127,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=132219</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3891,7 +4137,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr">
         <is>
           <t>valid_to_wrong</t>
@@ -3902,11 +4147,23 @@
           <t>Có cạnh 'Văn bản được thay thế' trỏ vào NĐ 114/2018/NĐ-CP nhưng valid_to rỗng; id cũ vilextime:T1:provision:b8918060-2d46-11f1-8ed9-293a0f03a912:2018-09-05: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S44" t="inlineStr"/>
-      <c r="T44" t="inlineStr"/>
-      <c r="U44" t="inlineStr"/>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr"/>
+      <c r="X44" s="2" t="inlineStr">
+        <is>
+          <t>114/2018/NĐ-CP · hiệu lực 2018-09-04 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 24. Cắm mốc chỉ giới xác định phạm vi bảo vệ đập thủy điện
+4. Phê duyệt phương án cắm mốc chỉ giới
+a) Chủ sở hữu đập, hồ chứa thủy điện nộp 01 bộ hồ sơ trực tiếp hoặc gửi qua đường bưu điện đến Ủy ban nhân dân cấp tỉnh nơi xây dựng đập. Hồ sơ gồm văn bản đề nghị phê duyệt và phương án cắm mốc chỉ giới;
+Trường hợp hồ sơ chưa hợp lệ, trong thời hạn 05 ngày làm việc, kể từ ngày nhận hồ sơ Ủy ban nhân dân cấp tỉnh thông báo bằng văn bản cho chủ sở hữu đập, hồ chứa thủy điện để hoàn chỉnh hồ sơ theo quy định;
+b) Trong thời hạn 25 ngày làm việc, kể từ ngày nhận đủ hồ sơ hợp lệ Ủy ban nhân dân cấp tỉnh có trách nhiệm tổ chức thẩm định;
+c) Trường hợp nội dung phương án cắm mốc chỉ giới phù hợp với quy định của pháp luật hiện hành và đặc điểm nơi xây dựng đập, trong thời hạn 05 ngày làm việc kể từ ngày tổ chức thẩm định, Ủy ban nhân dân cấp tỉnh có trách nhiệm phê duyệt. Trường hợp nội dung phương án cắm mốc chỉ giới không phù hợp với quy định của pháp luật hiện hành hoặc không phù hợp với đặc điểm nơi xây dựng đập, trong thời hạn 05 ngày làm việc kể từ ngày tổ chức thẩm định, Ủy ban nhân dân cấp tỉnh có trách nhiệm ban hành văn bản yêu cầu chủ sở hữu đập, hồ chứa thủy điện điều chỉnh, bổ sung phương án cắm mốc chỉ giới;
+d) Đối với đập có phạm vi bảo vệ thuộc địa bàn một huyện, Ủy ban nhân dân cấp tỉnh xem xét quyết định phân cấp cho Ủy ban nhân dân cấp huyện nơi xây dựng đập phê duyệt.</t>
+        </is>
+      </c>
+      <c r="Y44" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3959,9 +4216,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=23099</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -3972,18 +4226,29 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:bcd427a2-df46-11f0-9393-9f1aa228ec14#k1#c:2001-10-21: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
-      <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
+      <c r="X45" s="2" t="inlineStr">
+        <is>
+          <t>71/2001/NĐ-CP · hiệu lực 2001-10-20 → 2006-10-08 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 12. Quỹ phát triển nhà ở
+1. Căn cứ nhu cầu, điều kiện và chương trình phát triển nhà ở của địa phương, Chủ tịch Uỷ ban nhân dân cấp tỉnh có thể quyết định thành lập Quỹ phát triển nhà ở để huy động các nguồn vốn phục vụ đầu tư phát triển nhà ở trên địa bàn theo quy định như sau:
+a) Quỹ phát triển nhà ở được hình thành từ các nguồn: ngân sách nhà nước (tiền bán nhà ở thuộc sở hữu Nhà nước, khấu hao cơ bản trích từ tiền cho thuê nhà ở thuộc sở hữu Nhà nước, tiền sử dụng đất ở và các nguồn ngân sách khác nếu có); tiền huy động, tiền gửi của người có nhu cầu mua nhà ở, tiền hỗ trợ, tiền đóng góp tự nguyện của các tổ chức, cá nhân trong và ngoài nước và các hình thức huy động vốn hợp pháp khác theo quy định của pháp luật;
+b) Qũy phát triển nhà ở hoạt động theo nguyên tắc bảo toàn vốn và bù đắp chi phí theo Điều lệ do Bộ trưởng Bộ Tài chính quy định, sau khi thống nhất với Bộ trưởng Bộ Xây dựng;
+c) Quỹ phát triển nhà ở được sử dụng vào các mục đích sau:
+Cho các doanh nghiệp trong nước quy định tại khoản 1 Điều 3 Nghị định này vay với lãi suất thấp để đầu tư xây dựng các dự án nhà ở được ưu đãi;
+Cho các đối tượng hưởng lương từ ngân sách nhà nước vay với lãi suất thấp để mua nhà ở;
+Cho các doanh nghiệp trong nước vay với điều kiện tín dụng thuận lợi để đầu tư xây dựng các dự án nhà ở.</t>
+        </is>
+      </c>
+      <c r="Y45" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4036,9 +4301,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=155496</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4049,18 +4311,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:d20598e6-df59-11f0-a9f3-71e4d6f8e635#k7:2021-01-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr"/>
-      <c r="T46" t="inlineStr"/>
-      <c r="U46" t="inlineStr"/>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
+      <c r="X46" s="2" t="inlineStr">
+        <is>
+          <t>63/2020/TT-BCA · hiệu lực 2021-01-01 → 2025-01-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 9. Khám nghiệm hiện trường
+7. Sau khi khám nghiệm hiện trường, cán bộ Cảnh sát giao thông được phân công điều tra, xác minh, giải quyết vụ tai nạn giao thông phải có Báo cáo kết quả khám nghiệm hiện trường vụ tai nạn giao thông đường bộ theo mẫu số 07/TNĐB ban hành theo Thông tư này và đề xuất các biện pháp điều tra, xác minh, giải quyết tiếp theo.</t>
+        </is>
+      </c>
+      <c r="Y46" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4113,9 +4380,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=44169</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4126,7 +4390,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr">
         <is>
           <t>valid_to_wrong</t>
@@ -4137,11 +4400,18 @@
           <t>Luật Tổ chức TAND 62/2014/QH13 đã bị Luật 34/2024/QH15 thay thế từ 01/01/2025; valid_to vẫn rỗng; id cũ vilextime:T1:provision:d93e71d8-df44-11f0-8872-818f0d72bc1d:2015-06-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr"/>
-      <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr"/>
+      <c r="X47" s="2" t="inlineStr">
+        <is>
+          <t>62/2014/QH13 · hiệu lực 2015-06-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 74. Nhiệm kỳ của Thẩm phán
+Nhiệm kỳ đầu của các Thẩm phán là 05 năm; trường hợp được bổ nhiệm lại hoặc được bổ nhiệm vào ngạch Thẩm phán khác thì nhiệm kỳ tiếp theo là 10 năm.</t>
+        </is>
+      </c>
+      <c r="Y47" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4169,7 +4439,6 @@
           <t>2011-07-30 (giua_khoang)</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>4.2. Trong số các hạng mục phải kiểm tra chất lượng về môi trường cần đặc biệt chú ý kiểm tra các hệ thống chống thấm, hệ thống thu gom và xử lý nước rác, hệ thống thu gom, đánh giá và khử biogas cũng như hệ thống giếng quan trắc nước dưới đất, các trạm quan trắc nước mặt. Công tác kiểm tra phải được tiến hành cả ở hiện trường và trong phòng thí nghiệm, đúng hạng mục và phù hợp với từng thời điểm cần thiết nhằm đảm bảo sao cho những vật liệu và thiết bị sử dụng trong BCL đáp ứng các tiêu chuẩn Việt Nam về môi trường (TCVN).</t>
@@ -4190,9 +4459,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=23306</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4203,7 +4469,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -4214,11 +4479,17 @@
           <t>Đáp án là mục 4.2 nhưng citation là 'Khoản 4'; id cũ vilextime:T1:provision:dfeea17c-e16c-11f0-ab71-f3424eab00a5:2001-02-03: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr"/>
-      <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
+      <c r="X48" s="2" t="inlineStr">
+        <is>
+          <t>01/2001/TTLT/BKHCNMT-BXD · hiệu lực 2001-02-02 → 2019-08-15 · lúc thu thập: Hết hiệu lực toàn bộ
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y48" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4271,9 +4542,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=105944</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4284,18 +4552,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Theo quy định về phối hợp trao đổi thông tin bảo đảm an ninh hàng không dân dụng, thông tin về tình hình nước ngoài nào thuộc nội dung phải trao đổi?»; nhãn cũ khong_dat question_ambiguous: 'Thông tin về tình hình nước ngoài' cũng khớp khoản 3 (tội phạm, khủng bố quốc tế) và khoản 6 (xu hướng ngành hàng không các nước)). Câu hỏi chốt tình hình an ninh, chính trị các nước có đường bay; id cũ vilextime:T1:provision:e1d96590-df4a-11f0-b9c1-975d55408b6a:2016-06-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S49" t="inlineStr"/>
-      <c r="T49" t="inlineStr"/>
-      <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr"/>
+      <c r="X49" s="2" t="inlineStr">
+        <is>
+          <t>07/2016/TTTL-BGTVT-BCA-BQP · hiệu lực 2016-06-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 4. Nội dung thông tin trao đổi
+4. Tình hình an ninh, chính trị các nước, khu vực có đường bay đi, đến, bay qua Việt Nam.</t>
+        </is>
+      </c>
+      <c r="Y49" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4348,9 +4621,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=159420</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4361,18 +4631,33 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Theo quy định về hồ sơ đồ án quy hoạch xây dựng, bản đồ tổng hợp đường dây, đường ống kỹ thuật phải được thể hiện trên nền bản đồ nào và theo tỷ lệ nào?»; nhãn cũ khong_dat question_ambiguous: Câu hỏi không nêu loại đồ án; Điều 10, 12, 27, 29, 36 cùng có mục 'Bản đồ tổng hợp đường dây, đường ống kỹ thuật' với nền bản đồ/tỷ lệ khác nhau). Đã nêu đồ án quy hoạch phân khu đô thị (Điều 10); id cũ vilextime:T1:provision:ebf45422-df54-11f0-b907-ef5b243581fd#k1#h:2023-01-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr"/>
-      <c r="T50" t="inlineStr"/>
-      <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr"/>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>04/2022/TT-BXD · hiệu lực 2023-01-01 → 2025-07-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 10. Nội dung hồ sơ đồ án quy hoạch phân khu đô thị
+1. Thành phần bản vẽ bao gồm:
+a) Sơ đồ vị trí và giới hạn khu đất: Vị trí, phạm vi ranh giới lập quy hoạch, thể hiện mối quan hệ giữa khu vực lập quy hoạch với các khu vực khác trong đô thị. Bản vẽ hiện trên sơ đồ hướng phát triển không gian và bản đồ quy hoạch sử dụng đất đô thị theo các giai đoạn quy hoạch ở tỷ lệ thích hợp.
+b) Bản đồ hiện trạng sử dụng đất và kiến trúc, cảnh quan: Hiện trạng chức năng sử dụng đất theo quy định tại Phụ lục V của Thông tư này và các chỉ tiêu sử dụng đất; hiện trạng kiến trúc cảnh quan, hệ thống hạ tầng xã hội (giáo dục, y tế, văn hóa, thể dục thể thao, thương mại, cây xanh, nhà ở,...), các khu vực bảo vệ di tích, di sản, danh lam thắng cảnh. Bản vẽ thể hiện trên nền bản đồ địa hình tỷ lệ 1/2.000 hoặc 1/5.000.
+c) Các bản đồ hiện trạng hệ thống hạ tầng kỹ thuật và bảo vệ môi trường: Giao thông, cấp điện và chiếu sáng đô thị, thông tin liên lạc, cấp nước, cao độ nền và thoát nước mưa, thoát nước thải; quản lý chất thải rắn, nghĩa trang và môi trường; công trình hạ tầng kỹ thuật khác. Bản đồ thể hiện trên nền bản đồ địa hình tỷ lệ 1/2.000 hoặc 1/5.000.
+d) Bản đồ quy hoạch tổng mặt bằng sử dụng đất: Xác định quy mô diện tích, dân số và chỉ tiêu sử dụng đất quy hoạch đối với từng ô phố trong khu vực lập quy hoạch theo quy định tại Phụ lục V của Thông tư này; khoảng lùi công trình đối với các trục đường trong khu vực lập quy hoạch; vị trí, quy mô công trình ngầm. Xác định các đơn vị ở; vị trí, quy mô của hệ thống hạ tầng xã hội cấp đô thị trở lên (nếu có) và cấp đơn vị ở trong khu vực. Bản vẽ thể hiện trên nền bản đồ địa hình tỷ lệ 1/2.000 hoặc 1/5.000.
+đ) Sơ đồ tổ chức không gian kiến trúc cảnh quan: Bản vẽ thể hiện trên nền bản đồ địa hình tỷ lệ 1/2.000 hoặc 1/5.000.
+e) Bản đồ quy hoạch hệ thống công trình giao thông và chỉ giới đường đỏ, chỉ giới xây dựng đến cấp đường khu vực đối với bản vẽ tỷ lệ 1/5.000 hoặc đ ường phân khu vực đối với bản vẽ 1/2.000; vị trí, quy mô bến, bãi đỗ xe (trên cao, trên mặt đất và ngầm); tuyến và ga tàu điện ngầm ; hào và tuynel kỹ thuật. Bản vẽ thể hiện trên nền bản đồ quy hoạch tổng mặt bằng sử dụng đất kết hợp bản đồ địa hình tỷ lệ 1/2.000 hoặc 1/5.000.
+g) Các bản đồ quy hoạch hệ thống công trình hạ tầng kỹ thuật theo từng chuyên ngành: Chuẩn bị kỹ thuật, cấp nước, cấp năng lượng và chiếu sáng, thoát nước thải và xử lý chất thải rắn, hạ tầng viễn thông thụ động và công trình hạ tầng kỹ thuật khác. Thể hiện trên nền bản đồ quy hoạch tổng mặt bằng sử dụng đất kết hợp bản đồ địa hình tỷ lệ 1/2.000 hoặc 1/5.000.
+h) Bản đồ tổng hợp đường dây, đường ống kỹ thuật. Bản vẽ thể hiện trên nên bản đồ quy hoạch tổng mặt bằng sử dụng đất kết hợp bản đồ địa hình tỷ lệ 1/2.000 hoặc 1/5.000.
+i) Bản vẽ xác định các khu vực xây dựng công trình ngầm : Các công trình công cộng ngầm , các công trình cao tầng có xây dựng tầng hầm (nếu có). Bản vẽ thể hiện theo tỷ lệ thích hợp trên nền bản đồ quy hoạch tổng mặt bằng sử dụng đất , bản đồ tổng hợp đường dây, đường ống kỹ thuật kết hợp bản đồ địa hình.
+k) Các bản vẽ thiết kế đô thị: Thể hiện theo quy định tại Thông tư số 06/2013/TT-BXD .</t>
+        </is>
+      </c>
+      <c r="Y50" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4425,9 +4710,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=13699</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4438,7 +4720,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr">
         <is>
           <t>citation_path_wrong</t>
@@ -4449,11 +4730,17 @@
           <t>Mục 1.2.b bị ghi thành 'Điểm b Khoản 1' (lead_in '1. 2 Kiểm kê ...'); id cũ vilextime:T1:provision:ee6092ba-eb76-11f0-a704-8938278d801d:2007-05-29: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S51" t="inlineStr"/>
-      <c r="T51" t="inlineStr"/>
-      <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr"/>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>25/2007/TT-BTC · hiệu lực 2007-05-28 → 2010-05-05 · lúc thu thập: Hết hiệu lực toàn bộ
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y51" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4506,9 +4793,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=139885</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4519,18 +4803,27 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:f2798c00-22ab-11f1-b463-8f1119e7a6db:2021-01-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S52" t="inlineStr"/>
-      <c r="T52" t="inlineStr"/>
-      <c r="U52" t="inlineStr"/>
-      <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr"/>
+      <c r="X52" s="2" t="inlineStr">
+        <is>
+          <t>54/2019/QH14 · hiệu lực 2021-01-01 → nay · lúc thu thập: Hết hiệu lực một phần
+Điều 41. Nội dung quản trị công ty áp dụng đối với công ty đại chúng
+2. Việc triệu tập, tổ chức họp Đại hội đồng cổ đông tuân thủ các quy định sau đây:
+a) Hội đồng quản trị, Ban kiểm soát, người triệu tập họp Đại hội đồng cổ đông phải tuân thủ đầy đủ trình tự, thủ tục về triệu tập họp Đại hội đồng cổ đông theo quy định của Luật Doanh nghiệp, Điều lệ công ty và Quy chế nội bộ về quản trị công ty; bố trí địa điểm, thời gian hợp lý để các cổ đông tham dự họp Đại hội đồng cổ đông;
+b) Công ty đại chúng quy định tại Quy chế nội bộ về quản trị công ty việc áp dụng công nghệ thông tin hiện đại để cổ đông có thể tham dự và phát biểu ý kiến tại cuộc họp Đại hội đồng cổ đông thông qua họp trực tuyến, bỏ phiếu điện tử hoặc hình thức điện tử khác theo quy định của Luật Doanh nghiệp và Điều lệ công ty;
+c) Công ty đại chúng phải mời đại diện tổ chức kiểm toán được chấp thuận thực hiện kiểm toán Báo cáo tài chính năm của công ty dự họp Đại hội đồng cổ đông thường niên trong trường hợp Báo cáo kiểm toán báo cáo tài chính năm của công ty có các khoản ngoại trừ trọng yếu;
+d) Tuân thủ các quy định khác của pháp luật và Điều lệ công ty.</t>
+        </is>
+      </c>
+      <c r="Y52" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4583,9 +4876,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=164267</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4596,7 +4886,6 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr">
         <is>
           <t>citation_path_wrong,lead_in_wrong,group_wrong</t>
@@ -4612,10 +4901,57 @@
           <t>"Điều 4a. Cách thức gửi, nhận hồ sơ..."</t>
         </is>
       </c>
-      <c r="T53" t="inlineStr"/>
-      <c r="U53" t="inlineStr"/>
-      <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
+      <c r="X53" s="2" t="inlineStr">
+        <is>
+          <t>16/2023/TT-NHNN · hiệu lực 2024-07-01 → 2026-03-01 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 4. Nội dung chứng thư số
+1. Tên tổ chức cung cấp dịch vụ chữ ký số.
+2. Tên của thuê bao.
+3. Số hiệu (Serial Number) của chứng thư số.
+4. Thời hạn có hiệu lực của chứng thư số.
+5. Khóa công khai của thuê bao.
+6. Chữ ký số của tổ chức cung cấp dịch vụ chữ ký số.
+7. Các hạn chế về mục đích, phạm vi sử dụng của chứng thư số.
+8. Các hạn chế về trách nhiệm pháp lý của tổ chức cung cấp dịch vụ chữ ký số.
+9. Thuật toán mật mã.
+10. Các nội dung cần thiết khác theo quy định của Bộ Thông tin và Truyền thông."
+5. Sửa đổi, bổ sung Điều 4a Thông tư 28/2015/TT-NHNN (đã được sửa đổi, bổ sung bởi khoản 4 Điều 1 Thông tư 10/2020/TT-NHNN) như sau:
+"Điều 4a. Cách thức gửi, nhận hồ sơ, văn bản, báo cáo liên quan đến dịch vụ chứng thực chữ ký số và kết quả xử lý
+1. Tổ chức quản lý thuê bao gửi hồ sơ, văn bản, báo cáo liên quan đến chứng thư số và dịch vụ chứng thực chữ ký số đến Ngân hàng Nhà nước (Cục Công nghệ thông tin) thông qua một trong các phương thức sau:
+a) Phương thức điện tử qua Hệ thống dịch vụ công;
+b) Văn bản giấy nộp trực tiếp tại Bộ phận Một cửa hoặc gửi qua dịch vụ bưu chính
+c) Văn bản điện tử gửi qua hệ thống Quản lý văn bản và điều hành của Ngân hàng Nhà nước (áp dụng đối với các đơn vị thuộc Ngân hàng Nhà nước). Ngân hàng Nhà nước (Cục Công nghệ thông tin) chỉ tiếp nhận, xử lý văn bản giấy và văn bản điện tử gửi qua hệ thống Quản lý văn bản và điều hành của Ngân hàng Nhà nước trong các trường hợp sau đây:
+- Hệ thống dịch vụ công gặp sự cố không thể hoạt động được;
+- Tổ chức quản lý thuê bao chưa được cấp chứng thư số có nghiệp vụ dịch vụ công hoặc chứng thư số hết hiệu lực hoặc thiết bị lưu khóa bí mật của thuê bao bị hỏng.
+2. Gửi hồ sơ, văn bản, báo cáo liên quan đến chứng thư số và dịch vụ chứng thực chữ ký số Ngân hàng Nhà nước
+a) Trường hợp gửi hồ sơ, văn bản, báo cáo bản giấy: Tổ chức quản lý thuê bao có quyền lựa chọn gửi bản gốc hoặc bản sao được cấp từ sổ gốc hoặc bản sao có chứng thực hoặc bản sao kèm xuất trình bản chính để đối chiếu.
+b) Trường hợp gửi hồ sơ, văn bản, báo cáo điện tử: Các hồ sơ, văn bản, báo cáo (trừ các văn bản, báo cáo là các Phụ lục của Thông tư này đã được chuyển đổi thành các biểu mẫu điện tử trên Hệ thống dịch vụ công) gửi qua Hệ thống dịch vụ công, tổ chức quản lý thuê bao gửi bản điện tử được số hóa từ bản gốc (tập tin định dạng PDF) và được người có thẩm quyền của tổ chức quản lý thuê bao ký số sử dụng chứng thư số của CA-NHNN.
+3. Cục Công nghệ thông tin gửi thông báo kết quả xử lý, lý do từ chối trong trường hợp hồ sơ không được chấp thuận đến tổ chức quản lý thuê bao bằng phương thức điện tử qua Hệ thống dịch vụ công. Trường hợp Hệ thống dịch vụ công gặp sự cố, thông báo kết quả được gửi đến tổ chức quản lý thuê bao qua dịch vụ bưu chính hoặc địa chỉ thư điện tử của thuê bao và cá nhân hoặc bộ phận đầu mối phụ trách quản lý chứng thư số của tổ chức quản lý thuê bao."
+6. Sửa đổi, bổ sung Điều 4b Thông tư 28/2015/TT-NHNN (đã được sửa đổi, bổ sung bởi khoản 5 Điều 1 Thông tư 10/2020/TT-NHNN) như sau:
+"Điều 4b. Thiết bị lưu khóa bí mật của thuê bao
+1. Cục Công nghệ thông tin có trách nhiệm hướng dẫn về chủng loại, thông số kỹ thuật thiết bị lưu khóa bí mật của thuê bao phù hợp với hệ thống chứng thực chữ ký số Ngân hàng Nhà nước và tình hình phát triển công nghệ.
+2. Cục Công nghệ thông tin cung cấp thiết bị lưu khóa bí mật cho các đơn vị hành chính thuộc Ngân hàng Nhà nước. Các đơn vị sự nghiệp thuộc Ngân hàng Nhà nước và các tổ chức quản lý thuê bao khác tự trang bị thiết bị lưu khóa bí mật theo đúng hướng dẫn của Cục Công nghệ thông tin.
+3. Việc gửi, nhận thiết bị lưu khóa bí mật giữa Cục Công nghệ thông tin và các đơn vị hành chính thuộc Ngân hàng Nhà nước được thực hiện bằng phương thức trực tiếp hoặc thông qua dịch vụ bưu chính."
+7. Sửa đổi, bổ sung Điều 5 Thông tư 28/2015/TT-NHNN (đã được sửa đổi, bổ sung bởi khoản 6 Điều 1 Thông tư 10/2020/TT-NHNN) như sau:
+"Điều 5. Cấp, bổ sung nghiệp vụ chứng thư số
+1. Khi có nhu cầu cấp chứng thư số hoặc bổ sung nghiệp vụ, tổ chức quản lý thuê bao gửi 01 (một) bộ hồ sơ bao gồm:
+a) Cấp, bổ sung nghiệp vụ chứng thư số cho cá nhân là người có thẩm quyền: - Giấy đề nghị cấp, bổ sung nghiệp vụ chứng thư số cho cá nhân theo Phụ lục 01 ban hành kèm theo Thông tư này; - Quyết định bổ nhiệm của người có thẩm quyền khi đề nghị cấp mới chứng thư số (đối với cơ quan nhà nước).
+b) Cấp, bổ sung nghiệp vụ chứng thư số cho cá nhân là người được người có thẩm quyền ủy quyền:
+- Giấy đề nghị cấp, bổ sung nghiệp vụ chứng thư số cho cá nhân theo Phụ lục 01 ban hành kèm theo Thông tư này;
+- Quyết định bổ nhiệm của người có thẩm quyền khi đề nghị cấp mới chứng thư số (đối với cơ quan nhà nước);
+- Văn bản ủy quyền của người có thẩm quyền cho cá nhân được cấp chứng thư số hoặc bổ sung nghiệp vụ chứng thư số, nêu rõ người được ủy quyền được phép đại diện cho tổ chức ký duyệt hồ sơ, văn bản, tài liệu, báo cáo, giao dịch trên hệ thống thông tin tương ứng với nghiệp vụ của chứng thư số đề nghị cấp. Người được ủy quyền không được ủy quyền lại cho người khác thực hiện
+c) Cấp, bổ sung nghiệp vụ chứng thư số cho tổ chức:
+Giấy đề nghị cấp, bổ sung nghiệp vụ chứng thư số cho tổ chức theo Phụ lục 02 ban hành kèm theo Thông tư này.
+2. Trường hợp chứng thư số đã được cấp và còn hiệu lực, được tổ chức quản lý thuê bao đề nghị bổ sung nghiệp vụ chứng thư số, Cục Công nghệ thông tin thực hiện bổ sung nghiệp vụ cho chứng thư số hiện có của thuê bao.
+3. Trường hợp cấp chứng thư số sau khi chứng thư số cũ hết hiệu lực hoặc chứng thư số đã bị thu hồi, thuê bao có nhu cầu tiếp tục sử dụng thì thực hiện thủ tục cấp mới chứng thư số theo quy định tại khoản 1 Điều này.
+4. Thời hạn giải quyết và kết quả thực hiện Trong thời hạn 03 ngày làm việc kể từ ngày nhận được hồ sơ đề nghị cấp chứng thư số hợp lệ, Cục Công nghệ thông tin thực hiện cấp chứng thư số hoặc bổ sung nghiệp vụ chứng thư số cho thuê bao, gửi thông báo cấp chứng thư số và mã kích hoạt chứng thư số đến địa c</t>
+        </is>
+      </c>
+      <c r="Y53" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4668,9 +5004,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=91876</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4681,18 +5014,23 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
           <t>id cũ vilextime:T1:provision:fcda0fa4-e14b-11f0-9ac4-238e516e6c2b#k4:2016-01-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S54" t="inlineStr"/>
-      <c r="T54" t="inlineStr"/>
-      <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>52/2015/QĐ-TTg · hiệu lực 2016-01-01 → 2018-01-23 · lúc thu thập: Hết hiệu lực toàn bộ
+Điều 32. Hiệu lực thi hành
+4. Trường hợp cần điều hành linh hoạt hoạt động thương mại biên giới phù hợp với điều kiện kinh tế - xã hội của từng địa phương và trong từng thời kỳ, Thủ tướng Chính phủ xem xét quyết định việc điều chỉnh hoạt động mua bán hàng hóa qua biên giới của thương nhân và cư dân biên giới trên cơ sở đề nghị của Bộ Công Thương.</t>
+        </is>
+      </c>
+      <c r="Y54" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4720,7 +5058,6 @@
           <t>2001-11-28 (giua_khoang)</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>5. Thông tư này có hiệu lực sau 15 ngày, kể từ ngày ký.</t>
@@ -4741,9 +5078,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=22671</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4754,18 +5088,22 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
           <t>Điều khoản hiệu lực của chính thông tư, không phải quy phạm nội dung — cân nhắc loại khỏi T1; id cũ vilextime:T1:provision:fe20558c-e180-11f0-a914-ddbb65539df3:2001-10-04: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr"/>
-      <c r="T55" t="inlineStr"/>
-      <c r="U55" t="inlineStr"/>
-      <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr"/>
+      <c r="X55" s="2" t="inlineStr">
+        <is>
+          <t>07/2001/TT-BCA (V19) · hiệu lực 2001-10-03 → 2009-08-28 · lúc thu thập: Hết hiệu lực toàn bộ
+(không cắt được đoạn)</t>
+        </is>
+      </c>
+      <c r="Y55" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4818,9 +5156,6 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=163781</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
           <t>claude-opus-5-5</t>
@@ -4831,18 +5166,25 @@
           <t>dat</t>
         </is>
       </c>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr">
         <is>
           <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp đoạn rẽ từ đường bộ vào đường sắt ngắn hơn 10 mét, biển báo tại đường ngang phải được chọn và đặt như thế nào?»; nhãn cũ khong_dat question_ambiguous: Hỏi chung 'biển báo phải được chọn và đặt như thế nào' khi đoạn rẽ &lt; 10 m; điểm b cũng quy định biển phải đặt). Câu hỏi chốt 'căn cứ góc giao' nên chỉ khớp điểm a; id cũ vilextime:T1:provision:fe2ac128-eb6e-11f0-b2f9-27b4d1adb5b1:2023-12-02: spread_as_of (07/10) đổi as_of, cùng phiên bản và câu hỏi; nối lại 11/10</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr"/>
-      <c r="T56" t="inlineStr"/>
-      <c r="U56" t="inlineStr"/>
-      <c r="V56" t="inlineStr"/>
-      <c r="W56" t="inlineStr"/>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>29/2023/TT-BGTVT · hiệu lực 2023-12-01 → nay · lúc thu thập: Còn hiệu lực
+Điều 25. Yêu cầu đối với việc đặt biển báo hiệu trong trường hợp đường bộ liền kề và có đoạn rẽ vào đường sắt
+1. Khi chiều dài đoạn rẽ đến đường sắt nhỏ hơn 10 mét (m):
+a) Căn cứ góc giao của đường ngang, phải đặt biển "Nơi đường sắt giao vuông góc với đường bộ" hoặc "Nơi đường sắt giao không vuông góc với đường bộ" tại lề hai góc giao giữa đường bộ chạy gần với đoạn rẽ vào đường sắt;
+b) Căn cứ loại hình phòng vệ đường ngang phải đặt các biển "Giao nhau với đường sắt có rào chắn" hoặc "Giao nhau với đường sắt không có rào chắn" trên lề bên phải đường bộ chạy gần đường sắt. Khoảng cách các biển đến đoạn rẽ từ 40 mét (m) đến 240 mét (m).</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>(không có văn bản tác động)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>